<commit_message>
Refresh QA data and update validation and tvdiagnose scripts
</commit_message>
<xml_diff>
--- a/tte/qa/crossval_tte_vs_r.xlsx
+++ b/tte/qa/crossval_tte_vs_r.xlsx
@@ -21,7 +21,7 @@
     <t>Dataset: trial_example (503 patients, 48,400 person-periods)</t>
   </si>
   <si>
-    <t>Date:  7 Mar 2026</t>
+    <t>Date: 15 Mar 2026</t>
   </si>
   <si>
     <t>Config</t>
@@ -602,10 +602,10 @@
         <v>0.31377816200256348</v>
       </c>
       <c r="D7" s="5">
-        <v>0.31003560130675473</v>
+        <v>0.31003560130675462</v>
       </c>
       <c r="E7" s="6">
-        <v>0.0037425606958087498</v>
+        <v>0.0037425606958088609</v>
       </c>
       <c r="F7" t="s">
         <v>11</v>
@@ -662,10 +662,10 @@
         <v>0.4151584804058075</v>
       </c>
       <c r="D10" s="14">
-        <v>0.40880687009267708</v>
+        <v>0.40880687009267719</v>
       </c>
       <c r="E10" s="15">
-        <v>0.006351610313130418</v>
+        <v>0.006351610313130307</v>
       </c>
       <c r="F10" t="s">
         <v>15</v>
@@ -722,10 +722,10 @@
         <v>0.4151584804058075</v>
       </c>
       <c r="D13" s="23">
-        <v>0.40871870625843509</v>
+        <v>0.40871870625843459</v>
       </c>
       <c r="E13" s="24">
-        <v>0.0064397741473724013</v>
+        <v>0.0064397741473729009</v>
       </c>
       <c r="F13" t="s">
         <v>15</v>

</xml_diff>